<commit_message>
Change recon field keys
</commit_message>
<xml_diff>
--- a/data/cc.xlsx
+++ b/data/cc.xlsx
@@ -497,7 +497,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -509,7 +509,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>6</v>
@@ -521,7 +521,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="1"/>
       <c r="B4" s="2" t="s">
         <v>9</v>

</xml_diff>